<commit_message>
feat: show pictures, charts and text boxes in sheets
Read each sheet's drawing part and draw its anchored objects over the
grid: pictures as images, text boxes with their fill and text colors,
and charts as placeholders that show the chart title and point to Excel.

Drawings follow the same pane layout as cells, so one that crosses a
frozen row or column is split like in Excel. Sheets grow to include
drawings placed past the last used cell, and picture bytes are
transferred from the worker without copying.

The fixture workbook gains a Charts sheet built by the test writer,
which now writes drawing parts, PNG pictures and column charts.
</commit_message>
<xml_diff>
--- a/test/fixtures/sample.xlsx
+++ b/test/fixtures/sample.xlsx
@@ -9,12 +9,13 @@
     <sheet name="Data" sheetId="2" r:id="rId2"/>
     <sheet name="Hidden" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet name="No Grid" sheetId="4" r:id="rId4"/>
+    <sheet name="Charts" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t xml:space="preserve">Q3 Budget Overview</t>
   </si>
@@ -140,6 +141,9 @@
   </si>
   <si>
     <t xml:space="preserve">support@example.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drawings</t>
   </si>
 </sst>
 </file>
@@ -295,6 +299,397 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:t>Q3 revenue by region</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Q3</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Budget!$A$3:$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>North</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>South</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>East</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>West</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Central</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Online</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Budget!$C$3:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1385</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1012</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1060</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1598</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>802</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2650</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:crossAx val="2"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:crossAx val="1"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Q3</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Budget!$A$3:$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>North</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>South</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>East</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>West</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Central</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Online</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Budget!$C$3:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1385</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1012</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1060</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1598</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>802</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2650</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:crossAx val="2"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:r>
+                  <a:t>Thousands</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:crossAx val="1"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 3"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3048000" cy="609600"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="TextBox 4"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="BFBFBF"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Pictures, charts and text boxes</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>are drawn over the grid.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 5"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="914400" cy="457200"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 6"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
@@ -52609,4 +53004,21 @@
     <mergeCell ref="B2:D2"/>
   </mergeCells>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: show pictures, charts and text boxes in sheets (#10)
Pictures and text boxes are drawn where Excel anchors them, split across frozen panes like in Excel. Charts appear as placeholders with their title and a hint to open the file in Excel. Sheets grow to include drawings placed past the last used cell.
</commit_message>
<xml_diff>
--- a/test/fixtures/sample.xlsx
+++ b/test/fixtures/sample.xlsx
@@ -9,12 +9,13 @@
     <sheet name="Data" sheetId="2" r:id="rId2"/>
     <sheet name="Hidden" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet name="No Grid" sheetId="4" r:id="rId4"/>
+    <sheet name="Charts" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t xml:space="preserve">Q3 Budget Overview</t>
   </si>
@@ -140,6 +141,9 @@
   </si>
   <si>
     <t xml:space="preserve">support@example.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drawings</t>
   </si>
 </sst>
 </file>
@@ -295,6 +299,397 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:t>Q3 revenue by region</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Q3</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Budget!$A$3:$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>North</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>South</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>East</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>West</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Central</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Online</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Budget!$C$3:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1385</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1012</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1060</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1598</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>802</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2650</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:crossAx val="2"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:crossAx val="1"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Q3</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>Budget!$A$3:$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>North</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>South</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>East</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>West</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Central</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Online</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Budget!$C$3:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1385</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1012</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1060</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1598</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>802</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2650</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:crossAx val="2"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:r>
+                  <a:t>Thousands</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:crossAx val="1"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 3"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3048000" cy="609600"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="TextBox 4"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="BFBFBF"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr wrap="square" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Pictures, charts and text boxes</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>are drawn over the grid.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 5"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="914400" cy="457200"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 6"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
@@ -52609,4 +53004,21 @@
     <mergeCell ref="B2:D2"/>
   </mergeCells>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: apply conditional formatting in sheets
Evaluate each sheet's conditional formatting rules in the worker, once,
against the stored values, and draw the results over the cells' own
styles: fills, font colors and styles, color scales and data bars.

Supported rules are cell value comparisons (numbers, text, booleans and
single cell references, relative ones shifting with the range), text
matches, blanks and errors, top/bottom N or percent, above/below
average, duplicate and unique values, two- and three-color scales and
data bars. Priorities and stop-if-true work as in Excel. Rules that
need a formula engine and icon sets are skipped.

Colors adapt to dark themes like other fills; data bars are drawn
translucent so they read on both light and dark sheets. The fixture
workbook gains rules on the Budget and Data sheets, so the 100,000-row
check covers their cost as well.
</commit_message>
<xml_diff>
--- a/test/fixtures/sample.xlsx
+++ b/test/fixtures/sample.xlsx
@@ -296,6 +296,34 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -923,6 +951,37 @@
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:B8">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C8">
+    <cfRule type="dataBar" priority="3">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:D9">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E3:E8">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="season">
+      <formula>NOT(ISERROR(SEARCH("season",E3)))</formula>
+    </cfRule>
+  </conditionalFormatting>
 </worksheet>
 </file>
 
@@ -52963,6 +53022,19 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F2:F2001">
+    <cfRule type="top10" dxfId="1" priority="2" percent="1" rank="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G2001">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: apply conditional formatting in sheets (#11)
Highlight rules, color scales and data bars are evaluated once per sheet in the worker and drawn over the cells' own styles. Rules that need a formula engine and icon sets are skipped.
</commit_message>
<xml_diff>
--- a/test/fixtures/sample.xlsx
+++ b/test/fixtures/sample.xlsx
@@ -296,6 +296,34 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
@@ -923,6 +951,37 @@
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <conditionalFormatting sqref="B3:B8">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C8">
+    <cfRule type="dataBar" priority="3">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:D9">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E3:E8">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="season">
+      <formula>NOT(ISERROR(SEARCH("season",E3)))</formula>
+    </cfRule>
+  </conditionalFormatting>
 </worksheet>
 </file>
 
@@ -52963,6 +53022,19 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F2:F2001">
+    <cfRule type="top10" dxfId="1" priority="2" percent="1" rank="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G2001">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: spill text by alignment and fill styled rows and columns
Text that doesn't fit now spills the way Excel spills it: left-aligned
text to the right, right-aligned text to the left, and centered text
evenly to both sides. Center across selection centers text over the
following empty cells that share that alignment.

Rows and columns with a default style now show its fill across the
cells the file doesn't list, with row fills over column fills.

Merged cells and spilled text keep their outer right and bottom grid
lines instead of hiding them.
</commit_message>
<xml_diff>
--- a/test/fixtures/sample.xlsx
+++ b/test/fixtures/sample.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t xml:space="preserve">Q3 Budget Overview</t>
   </si>
@@ -141,6 +141,18 @@
   </si>
   <si>
     <t xml:space="preserve">support@example.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Right-aligned text spills left</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centered text spills to both sides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centered across B to D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A row style fills the whole row</t>
   </si>
   <si>
     <t xml:space="preserve">Drawings</t>
@@ -270,7 +282,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -295,6 +307,17 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0"/>
   </cellXfs>
   <dxfs count="3">
     <dxf>
@@ -53056,6 +53079,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="4" width="20" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1" style="20"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -53069,6 +53093,28 @@
       </c>
       <c r="C4" s="15" t="s">
         <v>41</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="F6" s="16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+    </row>
+    <row r="12" s="19" customFormat="1">
+      <c r="B12" s="19" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -53084,7 +53130,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: spill text by alignment and fill styled rows and columns (#12)
Text spills by its alignment (right-aligned to the left, centered to both sides), center across selection works, row and column default fills cover unlisted cells, and merged or spilled cells keep their outer grid lines.
</commit_message>
<xml_diff>
--- a/test/fixtures/sample.xlsx
+++ b/test/fixtures/sample.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t xml:space="preserve">Q3 Budget Overview</t>
   </si>
@@ -141,6 +141,18 @@
   </si>
   <si>
     <t xml:space="preserve">support@example.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Right-aligned text spills left</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centered text spills to both sides</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centered across B to D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A row style fills the whole row</t>
   </si>
   <si>
     <t xml:space="preserve">Drawings</t>
@@ -270,7 +282,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -295,6 +307,17 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0"/>
   </cellXfs>
   <dxfs count="3">
     <dxf>
@@ -53056,6 +53079,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="4" width="20" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1" style="20"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -53069,6 +53093,28 @@
       </c>
       <c r="C4" s="15" t="s">
         <v>41</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="F6" s="16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+    </row>
+    <row r="12" s="19" customFormat="1">
+      <c r="B12" s="19" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -53084,7 +53130,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: show the selected cell's formula in the status bar
Like Excel's formula bar, after the cell's value. Shared formulas, which
Excel stores once for a filled-down range, are moved to each cell's
position, array formulas show in braces across their range, and the
prefixes files keep on newer functions are dropped.
</commit_message>
<xml_diff>
--- a/test/fixtures/sample.xlsx
+++ b/test/fixtures/sample.xlsx
@@ -791,7 +791,7 @@
         <v>1385</v>
       </c>
       <c r="D3" s="5">
-        <f>C3/B3-1</f>
+        <f t="shared" ref="D3:D8" si="0">C3/B3-1</f>
         <v>0.117</v>
       </c>
       <c r="E3" t="s">
@@ -812,7 +812,7 @@
         <v>1012</v>
       </c>
       <c r="D4" s="5">
-        <f>C4/B4-1</f>
+        <f t="shared" si="0"/>
         <v>0.033</v>
       </c>
       <c r="E4" s="8" t="s">
@@ -833,7 +833,7 @@
         <v>1060</v>
       </c>
       <c r="D5" s="5">
-        <f>C5/B5-1</f>
+        <f t="shared" si="0"/>
         <v>-0.041</v>
       </c>
       <c r="E5" t="s">
@@ -854,7 +854,7 @@
         <v>1598</v>
       </c>
       <c r="D6" s="5">
-        <f>C6/B6-1</f>
+        <f t="shared" si="0"/>
         <v>0.117</v>
       </c>
       <c r="F6" s="7">
@@ -872,7 +872,7 @@
         <v>802</v>
       </c>
       <c r="D7" s="5">
-        <f>C7/B7-1</f>
+        <f t="shared" si="0"/>
         <v>0.055</v>
       </c>
       <c r="E7" t="s">
@@ -893,7 +893,7 @@
         <v>2650</v>
       </c>
       <c r="D8" s="5">
-        <f>C8/B8-1</f>
+        <f t="shared" si="0"/>
         <v>0.199</v>
       </c>
       <c r="E8" t="s">
@@ -916,6 +916,7 @@
         <v>8507</v>
       </c>
       <c r="D9" s="5">
+        <f>C9/B9-1</f>
         <v>0.101</v>
       </c>
       <c r="E9" s="9"/>

</xml_diff>

<commit_message>
feat: show the selected cell's formula in the status bar (#42)
Like Excel's formula bar, after the cell's value. Shared formulas, which
Excel stores once for a filled-down range, are moved to each cell's
position, array formulas show in braces across their range, and the
prefixes files keep on newer functions are dropped.
</commit_message>
<xml_diff>
--- a/test/fixtures/sample.xlsx
+++ b/test/fixtures/sample.xlsx
@@ -791,7 +791,7 @@
         <v>1385</v>
       </c>
       <c r="D3" s="5">
-        <f>C3/B3-1</f>
+        <f t="shared" ref="D3:D8" si="0">C3/B3-1</f>
         <v>0.117</v>
       </c>
       <c r="E3" t="s">
@@ -812,7 +812,7 @@
         <v>1012</v>
       </c>
       <c r="D4" s="5">
-        <f>C4/B4-1</f>
+        <f t="shared" si="0"/>
         <v>0.033</v>
       </c>
       <c r="E4" s="8" t="s">
@@ -833,7 +833,7 @@
         <v>1060</v>
       </c>
       <c r="D5" s="5">
-        <f>C5/B5-1</f>
+        <f t="shared" si="0"/>
         <v>-0.041</v>
       </c>
       <c r="E5" t="s">
@@ -854,7 +854,7 @@
         <v>1598</v>
       </c>
       <c r="D6" s="5">
-        <f>C6/B6-1</f>
+        <f t="shared" si="0"/>
         <v>0.117</v>
       </c>
       <c r="F6" s="7">
@@ -872,7 +872,7 @@
         <v>802</v>
       </c>
       <c r="D7" s="5">
-        <f>C7/B7-1</f>
+        <f t="shared" si="0"/>
         <v>0.055</v>
       </c>
       <c r="E7" t="s">
@@ -893,7 +893,7 @@
         <v>2650</v>
       </c>
       <c r="D8" s="5">
-        <f>C8/B8-1</f>
+        <f t="shared" si="0"/>
         <v>0.199</v>
       </c>
       <c r="E8" t="s">
@@ -916,6 +916,7 @@
         <v>8507</v>
       </c>
       <c r="D9" s="5">
+        <f>C9/B9-1</f>
         <v>0.101</v>
       </c>
       <c r="E9" s="9"/>

</xml_diff>